<commit_message>
3rd commit CRM : crm locators file created
</commit_message>
<xml_diff>
--- a/CRM_EPIC_0001.xlsx
+++ b/CRM_EPIC_0001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Universal_Framework_For_Web_And_Mobile_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0EBCE99-82AB-42E8-A007-9C5DDE1CD085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CD35C5-4545-45B9-A2B6-156B93BB9670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,112 +68,112 @@
 3. Verify that the CRM Admin successfully logs in and the main Dashboard page is displayed.</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The CRM Application is deployed and the Login URL is reachable (https://erp.qa.ethicalintelligent.com/crm/deals/CRM-DEAL-2026-00012#files)  and configured as base.url in config.properties.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid crm Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CRM Admin credentials (email and password) are configured in the config.properties file.</t>
+    </r>
+  </si>
+  <si>
+    <t>CRM Admin Login Url Should Be Accesiblle</t>
+  </si>
+  <si>
+    <t>Precondition[Regression]</t>
+  </si>
+  <si>
+    <t>Precondition[manual]</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Wait For Admin Login Page,wait_until_visible,,"crm.login_page.email_input_field"
 2. Enter User Name,type,administrator,"crm.login_page.email_input_field"
 3. Enter Password,type,erp@123,"crm.login_page.password_input_field"
 4. Click Login,click,,"crm.login_page.login_button"
-5.Wait For Dashboard,wait_until_visible,,"crm.dashboard.dashboard_siderbar_menu"
+5.Wait For Dashboard,wait_until_visible,,"crm.side_bar.dashboard_menu"
 6.Wait For View,wait,5000,
 </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The CRM Application is deployed and the Login URL is reachable (https://erp.qa.ethicalintelligent.com/crm/deals/CRM-DEAL-2026-00012#files)  and configured as base.url in config.properties.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid crm Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CRM Admin credentials (email and password) are configured in the config.properties file.</t>
-    </r>
-  </si>
-  <si>
-    <t>CRM Admin Login Url Should Be Accesiblle</t>
-  </si>
-  <si>
-    <t>Precondition[Regression]</t>
-  </si>
-  <si>
-    <t>Precondition[manual]</t>
   </si>
 </sst>
 </file>
@@ -562,10 +562,10 @@
         <v>7</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="J1" s="3"/>
     </row>
@@ -589,13 +589,13 @@
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>